<commit_message>
Documents (xls) modifications. See release notes for further info.
</commit_message>
<xml_diff>
--- a/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountUpdate_InstantProcess.xlsx
+++ b/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountUpdate_InstantProcess.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Deploy\IA\InterfacesGitHub\IA_CCBS_BANK_SIDE\AccountOther\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sw\Relational_Files\iApply\Interfaces\Interfaces_plus_allbanks\IA_CCBS_BANK_SIDE\AccountOther\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7658BD-42D5-4EB4-A823-E60FA0133964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EAFB136-F6C9-40A1-BFBA-CD35776E3D57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{68F28061-2ECD-4B0A-AB1D-3A449686159F}"/>
+    <workbookView xWindow="67080" yWindow="-5550" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{68F28061-2ECD-4B0A-AB1D-3A449686159F}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -530,7 +530,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -616,37 +616,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -721,46 +697,200 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent4" xfId="1" builtinId="42"/>
     <cellStyle name="60% - Accent4" xfId="2" builtinId="44"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <charset val="161"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -802,138 +932,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1215,149 +1213,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <charset val="161"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1372,32 +1227,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A6ACF92C-1104-4C93-8F8B-A938A4312D3B}" name="Table2" displayName="Table2" ref="B2:G34" totalsRowShown="0" headerRowDxfId="23" headerRowBorderDxfId="22" tableBorderDxfId="21" totalsRowBorderDxfId="20" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A6ACF92C-1104-4C93-8F8B-A938A4312D3B}" name="Table2" displayName="Table2" ref="B2:G34" totalsRowShown="0" headerRowDxfId="0" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:G31">
     <sortCondition ref="B3"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{85C05364-CF34-480B-84A9-1E752A61B8E7}" name="Seq" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{85C05364-CF34-480B-84A9-1E752A61B8E7}" name="Seq" dataDxfId="6" dataCellStyle="Normal"/>
     <tableColumn id="2" xr3:uid="{B74F6632-9589-464E-84C1-0830E8F1F8D8}" name="Description" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{9572A906-3602-4DBD-9459-262F500E1D9A}" name="iApply" dataDxfId="19" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{88CBB51C-2237-4EBC-90F4-9EFEDD4BEC32}" name="Data Type" dataDxfId="18" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{543BB0EE-DFCA-4B94-847F-73C897029E52}" name="Entities" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{2E373EFE-D19B-41E5-92FD-B165DCC3E8F5}" name="Notes" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{9572A906-3602-4DBD-9459-262F500E1D9A}" name="iApply" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{88CBB51C-2237-4EBC-90F4-9EFEDD4BEC32}" name="Data Type" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{543BB0EE-DFCA-4B94-847F-73C897029E52}" name="Entities" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{2E373EFE-D19B-41E5-92FD-B165DCC3E8F5}" name="Notes" dataDxfId="1" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F11F741B-5D22-4BBF-9B93-935C1585CBED}" name="Table22" displayName="Table22" ref="A1:F9" totalsRowShown="0" headerRowDxfId="17" headerRowBorderDxfId="16" tableBorderDxfId="15" totalsRowBorderDxfId="14" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F11F741B-5D22-4BBF-9B93-935C1585CBED}" name="Table22" displayName="Table22" ref="A1:F9" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:F9" xr:uid="{FE54AB27-2F61-427B-9D73-DA77A59601D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{F8F1211F-EA34-4B44-896A-D528AAFAE184}" name="Seq" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{03B9C3AE-C4F7-4512-A115-C772590AED2F}" name="Description" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{86EE5336-821C-4C56-8460-1456EB6E1740}" name="iApply" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{33764DB6-8011-4E1D-A09A-295251C6CCE7}" name="Data Type" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{AC1C2596-97D1-445C-B651-3EAD2A6C7064}" name="Entities" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{8FD2DAF4-1939-4C6D-BEB9-074AFC032812}" name="Notes" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{F8F1211F-EA34-4B44-896A-D528AAFAE184}" name="Seq" dataDxfId="16" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{03B9C3AE-C4F7-4512-A115-C772590AED2F}" name="Description" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{86EE5336-821C-4C56-8460-1456EB6E1740}" name="iApply" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{33764DB6-8011-4E1D-A09A-295251C6CCE7}" name="Data Type" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{AC1C2596-97D1-445C-B651-3EAD2A6C7064}" name="Entities" dataDxfId="12" dataCellStyle="Normal"/>
+    <tableColumn id="5" xr3:uid="{8FD2DAF4-1939-4C6D-BEB9-074AFC032812}" name="Notes" dataDxfId="11" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1701,20 +1556,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB8ACDA-C8F4-4728-9499-8B46BAA74AEA}">
   <dimension ref="B2:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.5546875" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.5703125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="17"/>
       <c r="C2" s="18" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="18" t="s">
         <v>10</v>
       </c>
@@ -1722,7 +1577,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="18" t="s">
         <v>12</v>
       </c>
@@ -1730,7 +1585,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="18" t="s">
         <v>13</v>
       </c>
@@ -1738,7 +1593,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="25" t="s">
         <v>20</v>
       </c>
@@ -1746,7 +1601,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="18" t="s">
         <v>14</v>
       </c>
@@ -1754,11 +1609,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="18"/>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="18" t="s">
         <v>16</v>
       </c>
@@ -1766,7 +1621,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="18" t="s">
         <v>18</v>
       </c>
@@ -1774,15 +1629,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="18"/>
       <c r="C11" s="19"/>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="18"/>
       <c r="C12" s="19"/>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="18" t="s">
         <v>19</v>
       </c>
@@ -1790,7 +1645,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="18"/>
       <c r="C14" s="19"/>
     </row>
@@ -1802,616 +1657,616 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03AC1DB5-1548-45C4-B0E5-7097191C5328}">
   <dimension ref="B1:G106"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1" style="2" customWidth="1"/>
-    <col min="2" max="2" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.21875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="67.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.109375" style="2"/>
+    <col min="2" max="2" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="67.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="4.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="31" t="s">
+    <row r="1" spans="2:7" ht="4.9000000000000004" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="23" t="s">
+      <c r="G2" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="32">
+    <row r="3" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="29">
         <v>1</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="28"/>
-    </row>
-    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="32">
+      <c r="G3" s="31"/>
+    </row>
+    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="29">
         <v>2</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="28"/>
-    </row>
-    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="32">
+      <c r="G4" s="31"/>
+    </row>
+    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="29">
         <v>3</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="26" t="s">
+      <c r="F5" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="28"/>
-    </row>
-    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="32">
+      <c r="G5" s="31"/>
+    </row>
+    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="29">
         <v>4</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="E6" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="28"/>
-    </row>
-    <row r="7" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="32">
+      <c r="G6" s="31"/>
+    </row>
+    <row r="7" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="29">
         <v>5</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="28"/>
-    </row>
-    <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="32">
+      <c r="G7" s="31"/>
+    </row>
+    <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="29">
         <v>6</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="28"/>
-    </row>
-    <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="32">
+      <c r="G8" s="31"/>
+    </row>
+    <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="29">
         <v>7</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="F9" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="28"/>
-    </row>
-    <row r="10" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="32">
+      <c r="G9" s="31"/>
+    </row>
+    <row r="10" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="29">
         <v>8</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="31" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="32">
+    <row r="11" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="29">
         <v>9</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="F11" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="28"/>
-    </row>
-    <row r="12" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="32">
+      <c r="G11" s="31"/>
+    </row>
+    <row r="12" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="29">
         <v>10</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="F12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="28"/>
-    </row>
-    <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="32">
+      <c r="G12" s="31"/>
+    </row>
+    <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="29">
         <v>11</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="26" t="s">
+      <c r="F13" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="28"/>
-    </row>
-    <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="32">
+      <c r="G13" s="31"/>
+    </row>
+    <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="29">
         <v>12</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="26" t="s">
+      <c r="F14" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G14" s="28"/>
-    </row>
-    <row r="15" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="32">
+      <c r="G14" s="31"/>
+    </row>
+    <row r="15" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="29">
         <v>13</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="F15" s="26" t="s">
+      <c r="F15" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G15" s="28"/>
-    </row>
-    <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="32">
+      <c r="G15" s="31"/>
+    </row>
+    <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="29">
         <v>14</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="28"/>
-    </row>
-    <row r="17" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="32">
+      <c r="G16" s="31"/>
+    </row>
+    <row r="17" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="29">
         <v>15</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F17" s="26" t="s">
+      <c r="F17" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G17" s="28"/>
-    </row>
-    <row r="18" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="32">
+      <c r="G17" s="31"/>
+    </row>
+    <row r="18" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="29">
         <v>16</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="F18" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G18" s="28"/>
-    </row>
-    <row r="19" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32">
+      <c r="G18" s="31"/>
+    </row>
+    <row r="19" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="29">
         <v>17</v>
       </c>
-      <c r="C19" s="26" t="s">
+      <c r="C19" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F19" s="26" t="s">
+      <c r="F19" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="28"/>
-    </row>
-    <row r="20" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="32">
+      <c r="G19" s="31"/>
+    </row>
+    <row r="20" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="29">
         <v>18</v>
       </c>
-      <c r="C20" s="26" t="s">
+      <c r="C20" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F20" s="26" t="s">
+      <c r="F20" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="28"/>
-    </row>
-    <row r="21" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="32">
+      <c r="G20" s="31"/>
+    </row>
+    <row r="21" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="29">
         <v>19</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="C21" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="26" t="s">
+      <c r="E21" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F21" s="26" t="s">
+      <c r="F21" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="28"/>
-    </row>
-    <row r="22" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="32">
+      <c r="G21" s="31"/>
+    </row>
+    <row r="22" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="29">
         <v>20</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="26" t="s">
+      <c r="D22" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="26" t="s">
+      <c r="E22" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F22" s="26" t="s">
+      <c r="F22" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G22" s="28"/>
-    </row>
-    <row r="23" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="32">
+      <c r="G22" s="31"/>
+    </row>
+    <row r="23" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="29">
         <v>21</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="D23" s="26" t="s">
+      <c r="D23" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F23" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="28"/>
-    </row>
-    <row r="24" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="32">
+      <c r="G23" s="31"/>
+    </row>
+    <row r="24" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="29">
         <v>22</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C24" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="26" t="s">
+      <c r="E24" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F24" s="26" t="s">
+      <c r="F24" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="28"/>
-    </row>
-    <row r="25" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="32">
+      <c r="G24" s="31"/>
+    </row>
+    <row r="25" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="29">
         <v>23</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C25" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="E25" s="26" t="s">
+      <c r="E25" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F25" s="26" t="s">
+      <c r="F25" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G25" s="28"/>
-    </row>
-    <row r="26" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="32">
+      <c r="G25" s="31"/>
+    </row>
+    <row r="26" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="29">
         <v>24</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D26" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="E26" s="26" t="s">
+      <c r="E26" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F26" s="26" t="s">
+      <c r="F26" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G26" s="28"/>
-    </row>
-    <row r="27" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="32">
+      <c r="G26" s="31"/>
+    </row>
+    <row r="27" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="29">
         <v>25</v>
       </c>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26" t="s">
+      <c r="C27" s="30"/>
+      <c r="D27" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F27" s="26" t="s">
+      <c r="F27" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G27" s="28"/>
-    </row>
-    <row r="28" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="32">
+      <c r="G27" s="31"/>
+    </row>
+    <row r="28" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="29">
         <v>26</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F28" s="26" t="s">
+      <c r="F28" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G28" s="28"/>
-    </row>
-    <row r="29" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="32">
+      <c r="G28" s="31"/>
+    </row>
+    <row r="29" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="29">
         <v>27</v>
       </c>
-      <c r="C29" s="26" t="s">
+      <c r="C29" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="26" t="s">
+      <c r="D29" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="E29" s="26" t="s">
+      <c r="E29" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F29" s="26" t="s">
+      <c r="F29" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G29" s="28"/>
-    </row>
-    <row r="30" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="32">
+      <c r="G29" s="31"/>
+    </row>
+    <row r="30" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="29">
         <v>28</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="26" t="s">
+      <c r="D30" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="26" t="s">
+      <c r="E30" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="26" t="s">
+      <c r="F30" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G30" s="28"/>
-    </row>
-    <row r="31" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="32">
+      <c r="G30" s="31"/>
+    </row>
+    <row r="31" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="29">
         <v>29</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="26" t="s">
+      <c r="D31" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="E31" s="26" t="s">
+      <c r="E31" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="F31" s="26" t="s">
+      <c r="F31" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="G31" s="28"/>
-    </row>
-    <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="37">
+      <c r="G31" s="31"/>
+    </row>
+    <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="33">
         <v>30</v>
       </c>
-      <c r="C32" s="33" t="s">
+      <c r="C32" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="E32" s="33" t="s">
+      <c r="E32" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="F32" s="33"/>
-      <c r="G32" s="34" t="s">
+      <c r="F32" s="34"/>
+      <c r="G32" s="35" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="37">
+    <row r="33" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B33" s="33">
         <v>31</v>
       </c>
-      <c r="C33" s="33" t="s">
+      <c r="C33" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="E33" s="33" t="s">
+      <c r="E33" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="F33" s="33"/>
-      <c r="G33" s="34" t="s">
+      <c r="F33" s="34"/>
+      <c r="G33" s="35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="38">
+    <row r="34" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="33">
         <v>32</v>
       </c>
-      <c r="C34" s="35" t="s">
+      <c r="C34" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="D34" s="35" t="s">
+      <c r="D34" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="E34" s="35" t="s">
+      <c r="E34" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="F34" s="35"/>
-      <c r="G34" s="36" t="s">
+      <c r="F34" s="34"/>
+      <c r="G34" s="35" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
       <c r="D35" s="7"/>
@@ -2419,7 +2274,7 @@
       <c r="F35" s="7"/>
       <c r="G35" s="8"/>
     </row>
-    <row r="36" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="5"/>
@@ -2427,7 +2282,7 @@
       <c r="F36" s="5"/>
       <c r="G36" s="6"/>
     </row>
-    <row r="37" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="5"/>
@@ -2435,7 +2290,7 @@
       <c r="F37" s="5"/>
       <c r="G37" s="6"/>
     </row>
-    <row r="38" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="5"/>
@@ -2443,19 +2298,19 @@
       <c r="F38" s="5"/>
       <c r="G38" s="6"/>
     </row>
-    <row r="39" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
       <c r="F39" s="5"/>
       <c r="G39" s="6"/>
     </row>
-    <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
       <c r="G40" s="6"/>
     </row>
-    <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="5"/>
@@ -2463,7 +2318,7 @@
       <c r="F41" s="5"/>
       <c r="G41" s="6"/>
     </row>
-    <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="7"/>
@@ -2471,7 +2326,7 @@
       <c r="F42" s="7"/>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="7"/>
@@ -2479,7 +2334,7 @@
       <c r="F43" s="7"/>
       <c r="G43" s="8"/>
     </row>
-    <row r="44" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="5"/>
@@ -2487,7 +2342,7 @@
       <c r="F44" s="5"/>
       <c r="G44" s="6"/>
     </row>
-    <row r="45" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="5"/>
@@ -2495,13 +2350,13 @@
       <c r="F45" s="5"/>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D46" s="5"/>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
       <c r="G46" s="6"/>
     </row>
-    <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="5"/>
@@ -2509,13 +2364,13 @@
       <c r="F47" s="5"/>
       <c r="G47" s="6"/>
     </row>
-    <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="6"/>
     </row>
-    <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="9"/>
@@ -2523,7 +2378,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="9"/>
     </row>
-    <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="9"/>
@@ -2531,7 +2386,7 @@
       <c r="F50" s="10"/>
       <c r="G50" s="9"/>
     </row>
-    <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
       <c r="D51" s="9"/>
@@ -2539,7 +2394,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="9"/>
     </row>
-    <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="9"/>
@@ -2547,7 +2402,7 @@
       <c r="F52" s="10"/>
       <c r="G52" s="9"/>
     </row>
-    <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="9"/>
@@ -2555,7 +2410,7 @@
       <c r="F53" s="10"/>
       <c r="G53" s="9"/>
     </row>
-    <row r="54" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="9"/>
@@ -2563,19 +2418,19 @@
       <c r="F54" s="10"/>
       <c r="G54" s="9"/>
     </row>
-    <row r="55" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D55" s="11"/>
       <c r="E55" s="11"/>
       <c r="F55" s="11"/>
       <c r="G55" s="12"/>
     </row>
-    <row r="56" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
       <c r="F56" s="5"/>
       <c r="G56" s="6"/>
     </row>
-    <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="5"/>
@@ -2583,7 +2438,7 @@
       <c r="F57" s="5"/>
       <c r="G57" s="6"/>
     </row>
-    <row r="58" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="13"/>
       <c r="C58" s="13"/>
       <c r="D58" s="11"/>
@@ -2591,7 +2446,7 @@
       <c r="F58" s="11"/>
       <c r="G58" s="12"/>
     </row>
-    <row r="59" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
       <c r="D59" s="11"/>
@@ -2599,7 +2454,7 @@
       <c r="F59" s="11"/>
       <c r="G59" s="12"/>
     </row>
-    <row r="60" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="11"/>
@@ -2607,7 +2462,7 @@
       <c r="F60" s="11"/>
       <c r="G60" s="12"/>
     </row>
-    <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="11"/>
@@ -2615,7 +2470,7 @@
       <c r="F61" s="11"/>
       <c r="G61" s="12"/>
     </row>
-    <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="14"/>
@@ -2623,7 +2478,7 @@
       <c r="F62" s="14"/>
       <c r="G62" s="15"/>
     </row>
-    <row r="63" spans="2:7" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:7" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="5"/>
@@ -2631,25 +2486,25 @@
       <c r="F63" s="5"/>
       <c r="G63" s="6"/>
     </row>
-    <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
       <c r="G64" s="6"/>
     </row>
-    <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
       <c r="G65" s="6"/>
     </row>
-    <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
       <c r="G66" s="6"/>
     </row>
-    <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
       <c r="D67" s="5"/>
@@ -2657,7 +2512,7 @@
       <c r="F67" s="5"/>
       <c r="G67" s="6"/>
     </row>
-    <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="11"/>
@@ -2665,7 +2520,7 @@
       <c r="F68" s="11"/>
       <c r="G68" s="12"/>
     </row>
-    <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="D69" s="11"/>
@@ -2673,49 +2528,49 @@
       <c r="F69" s="11"/>
       <c r="G69" s="12"/>
     </row>
-    <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
       <c r="G70" s="6"/>
     </row>
-    <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
       <c r="F71" s="5"/>
       <c r="G71" s="6"/>
     </row>
-    <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D72" s="11"/>
       <c r="E72" s="11"/>
       <c r="F72" s="11"/>
       <c r="G72" s="12"/>
     </row>
-    <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="5"/>
       <c r="G73" s="6"/>
     </row>
-    <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
       <c r="F74" s="5"/>
       <c r="G74" s="6"/>
     </row>
-    <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
       <c r="F75" s="5"/>
       <c r="G75" s="6"/>
     </row>
-    <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
       <c r="G76" s="6"/>
     </row>
-    <row r="77" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="5"/>
@@ -2723,7 +2578,7 @@
       <c r="F77" s="5"/>
       <c r="G77" s="6"/>
     </row>
-    <row r="78" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="5"/>
@@ -2731,7 +2586,7 @@
       <c r="F78" s="5"/>
       <c r="G78" s="6"/>
     </row>
-    <row r="79" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="5"/>
@@ -2739,127 +2594,127 @@
       <c r="F79" s="5"/>
       <c r="G79" s="6"/>
     </row>
-    <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
       <c r="G80" s="6"/>
     </row>
-    <row r="81" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
       <c r="G81" s="6"/>
     </row>
-    <row r="82" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
       <c r="F82" s="5"/>
       <c r="G82" s="6"/>
     </row>
-    <row r="83" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
       <c r="F83" s="5"/>
       <c r="G83" s="6"/>
     </row>
-    <row r="84" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
       <c r="G84" s="6"/>
     </row>
-    <row r="85" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D85" s="5"/>
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
       <c r="G85" s="6"/>
     </row>
-    <row r="86" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D86" s="5"/>
       <c r="E86" s="5"/>
       <c r="F86" s="5"/>
       <c r="G86" s="6"/>
     </row>
-    <row r="87" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
       <c r="F87" s="5"/>
       <c r="G87" s="6"/>
     </row>
-    <row r="88" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
       <c r="G88" s="6"/>
     </row>
-    <row r="89" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
       <c r="F89" s="5"/>
       <c r="G89" s="6"/>
     </row>
-    <row r="90" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
       <c r="F90" s="5"/>
       <c r="G90" s="6"/>
     </row>
-    <row r="91" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
       <c r="G91" s="6"/>
     </row>
-    <row r="92" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D92" s="5"/>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="6"/>
     </row>
-    <row r="93" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
       <c r="G93" s="6"/>
     </row>
-    <row r="94" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
       <c r="G94" s="6"/>
     </row>
-    <row r="95" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
       <c r="G95" s="6"/>
     </row>
-    <row r="96" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="5"/>
       <c r="G96" s="6"/>
     </row>
-    <row r="97" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
       <c r="G97" s="6"/>
     </row>
-    <row r="98" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
       <c r="G98" s="6"/>
     </row>
-    <row r="99" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
       <c r="G99" s="6"/>
     </row>
-    <row r="100" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="11"/>
@@ -2867,7 +2722,7 @@
       <c r="F100" s="11"/>
       <c r="G100" s="12"/>
     </row>
-    <row r="101" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="5"/>
@@ -2875,7 +2730,7 @@
       <c r="F101" s="5"/>
       <c r="G101" s="6"/>
     </row>
-    <row r="102" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
       <c r="D102" s="5"/>
@@ -2883,19 +2738,19 @@
       <c r="F102" s="5"/>
       <c r="G102" s="6"/>
     </row>
-    <row r="103" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
       <c r="G103" s="6"/>
     </row>
-    <row r="104" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D104" s="5"/>
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
       <c r="G104" s="6"/>
     </row>
-    <row r="105" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="16"/>
       <c r="C105" s="16"/>
       <c r="D105" s="5"/>
@@ -2903,7 +2758,7 @@
       <c r="F105" s="5"/>
       <c r="G105" s="6"/>
     </row>
-    <row r="106" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D106" s="5"/>
       <c r="E106" s="5"/>
       <c r="F106" s="5"/>
@@ -2911,7 +2766,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D31 D33:D1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2923,18 +2778,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DEFA5D-C6DF-4BEE-A0BF-87172BA2BD41}">
   <dimension ref="A1:F95"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" style="2" customWidth="1"/>
-    <col min="5" max="5" width="30.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="2"/>
+    <col min="5" max="5" width="30.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>8</v>
       </c>
@@ -2954,7 +2809,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20">
         <v>1</v>
       </c>
@@ -2972,7 +2827,7 @@
       </c>
       <c r="F2" s="27"/>
     </row>
-    <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="20">
         <v>2</v>
       </c>
@@ -2990,7 +2845,7 @@
       </c>
       <c r="F3" s="27"/>
     </row>
-    <row r="4" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20">
         <v>3</v>
       </c>
@@ -3008,7 +2863,7 @@
       </c>
       <c r="F4" s="27"/>
     </row>
-    <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="20">
         <v>4</v>
       </c>
@@ -3026,43 +2881,43 @@
       </c>
       <c r="F5" s="27"/>
     </row>
-    <row r="6" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="20">
         <v>5</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="F6" s="30"/>
-    </row>
-    <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F6" s="28"/>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="20">
         <v>6</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="30"/>
-    </row>
-    <row r="8" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F7" s="28"/>
+    </row>
+    <row r="8" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="20">
         <v>7</v>
       </c>
@@ -3080,25 +2935,25 @@
       </c>
       <c r="F8" s="27"/>
     </row>
-    <row r="9" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="20">
         <v>8</v>
       </c>
       <c r="B9" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="28" t="s">
         <v>97</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="28" t="s">
         <v>95</v>
       </c>
       <c r="F9" s="27"/>
     </row>
-    <row r="10" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="5"/>
@@ -3106,7 +2961,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="6"/>
     </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="5"/>
@@ -3114,7 +2969,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="6"/>
     </row>
-    <row r="12" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="7"/>
@@ -3122,13 +2977,13 @@
       <c r="E12" s="7"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="5"/>
@@ -3136,7 +2991,7 @@
       <c r="E14" s="5"/>
       <c r="F14" s="6"/>
     </row>
-    <row r="15" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="5"/>
@@ -3144,13 +2999,13 @@
       <c r="E15" s="5"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="6"/>
     </row>
-    <row r="17" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="5"/>
@@ -3158,31 +3013,31 @@
       <c r="E17" s="5"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="6"/>
     </row>
-    <row r="19" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="5"/>
@@ -3190,7 +3045,7 @@
       <c r="E22" s="5"/>
       <c r="F22" s="6"/>
     </row>
-    <row r="23" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="5"/>
@@ -3198,7 +3053,7 @@
       <c r="E23" s="5"/>
       <c r="F23" s="6"/>
     </row>
-    <row r="24" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="5"/>
@@ -3206,7 +3061,7 @@
       <c r="E24" s="5"/>
       <c r="F24" s="6"/>
     </row>
-    <row r="25" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="5"/>
@@ -3214,37 +3069,37 @@
       <c r="E25" s="5"/>
       <c r="F25" s="6"/>
     </row>
-    <row r="26" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="10"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="10"/>
       <c r="F27" s="9"/>
     </row>
-    <row r="28" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="10"/>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="10"/>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
       <c r="E30" s="10"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="9"/>
@@ -3252,13 +3107,13 @@
       <c r="E31" s="10"/>
       <c r="F31" s="9"/>
     </row>
-    <row r="32" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
       <c r="E32" s="11"/>
       <c r="F32" s="12"/>
     </row>
-    <row r="33" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="5"/>
@@ -3266,7 +3121,7 @@
       <c r="E33" s="5"/>
       <c r="F33" s="6"/>
     </row>
-    <row r="34" spans="1:6" s="13" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" s="13" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="5"/>
@@ -3274,7 +3129,7 @@
       <c r="E34" s="5"/>
       <c r="F34" s="6"/>
     </row>
-    <row r="35" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13"/>
       <c r="B35" s="13"/>
       <c r="C35" s="11"/>
@@ -3282,25 +3137,25 @@
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
     </row>
-    <row r="36" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
       <c r="E36" s="11"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="37" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
     </row>
-    <row r="38" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="12"/>
     </row>
-    <row r="39" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" s="14"/>
@@ -3308,25 +3163,25 @@
       <c r="E39" s="14"/>
       <c r="F39" s="15"/>
     </row>
-    <row r="40" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
       <c r="F40" s="6"/>
     </row>
-    <row r="41" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="6"/>
     </row>
-    <row r="42" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
       <c r="F42" s="6"/>
     </row>
-    <row r="43" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="5"/>
@@ -3334,19 +3189,19 @@
       <c r="E43" s="5"/>
       <c r="F43" s="6"/>
     </row>
-    <row r="44" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
       <c r="F44" s="6"/>
     </row>
-    <row r="45" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
     </row>
-    <row r="46" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="11"/>
@@ -3354,43 +3209,43 @@
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
     </row>
-    <row r="47" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
       <c r="F47" s="6"/>
     </row>
-    <row r="48" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
       <c r="F48" s="6"/>
     </row>
-    <row r="49" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C49" s="11"/>
       <c r="D49" s="11"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
     </row>
-    <row r="50" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
       <c r="F50" s="6"/>
     </row>
-    <row r="51" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
       <c r="F51" s="6"/>
     </row>
-    <row r="52" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
       <c r="F52" s="6"/>
     </row>
-    <row r="53" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="5"/>
@@ -3398,19 +3253,19 @@
       <c r="E53" s="5"/>
       <c r="F53" s="6"/>
     </row>
-    <row r="54" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
       <c r="F54" s="6"/>
     </row>
-    <row r="55" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
       <c r="F55" s="6"/>
     </row>
-    <row r="56" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="5"/>
@@ -3418,121 +3273,121 @@
       <c r="E56" s="5"/>
       <c r="F56" s="6"/>
     </row>
-    <row r="57" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
       <c r="F57" s="6"/>
     </row>
-    <row r="58" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
       <c r="F58" s="6"/>
     </row>
-    <row r="59" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C59" s="5"/>
       <c r="D59" s="5"/>
       <c r="E59" s="5"/>
       <c r="F59" s="6"/>
     </row>
-    <row r="60" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C60" s="5"/>
       <c r="D60" s="5"/>
       <c r="E60" s="5"/>
       <c r="F60" s="6"/>
     </row>
-    <row r="61" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C61" s="5"/>
       <c r="D61" s="5"/>
       <c r="E61" s="5"/>
       <c r="F61" s="6"/>
     </row>
-    <row r="62" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C62" s="5"/>
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
       <c r="F62" s="6"/>
     </row>
-    <row r="63" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
       <c r="E63" s="5"/>
       <c r="F63" s="6"/>
     </row>
-    <row r="64" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C64" s="5"/>
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
       <c r="F64" s="6"/>
     </row>
-    <row r="65" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C65" s="5"/>
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="6"/>
     </row>
-    <row r="66" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C66" s="5"/>
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="6"/>
     </row>
-    <row r="67" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C67" s="5"/>
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
       <c r="F67" s="6"/>
     </row>
-    <row r="68" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C68" s="5"/>
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
       <c r="F68" s="6"/>
     </row>
-    <row r="69" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
       <c r="F69" s="6"/>
     </row>
-    <row r="70" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C70" s="5"/>
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="6"/>
     </row>
-    <row r="71" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C71" s="5"/>
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
       <c r="F71" s="6"/>
     </row>
-    <row r="72" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
       <c r="F72" s="6"/>
     </row>
-    <row r="73" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="6"/>
     </row>
-    <row r="74" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
       <c r="F74" s="6"/>
     </row>
-    <row r="75" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
       <c r="F75" s="6"/>
     </row>
-    <row r="76" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="5"/>
@@ -3540,19 +3395,19 @@
       <c r="E76" s="5"/>
       <c r="F76" s="6"/>
     </row>
-    <row r="77" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C77" s="11"/>
       <c r="D77" s="11"/>
       <c r="E77" s="11"/>
       <c r="F77" s="12"/>
     </row>
-    <row r="78" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C78" s="5"/>
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
       <c r="F78" s="6"/>
     </row>
-    <row r="79" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="5"/>
@@ -3560,13 +3415,13 @@
       <c r="E79" s="5"/>
       <c r="F79" s="6"/>
     </row>
-    <row r="80" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="6"/>
     </row>
-    <row r="81" spans="1:6" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="5"/>
@@ -3574,7 +3429,7 @@
       <c r="E81" s="5"/>
       <c r="F81" s="6"/>
     </row>
-    <row r="82" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="16"/>
       <c r="B82" s="16"/>
       <c r="C82" s="5"/>
@@ -3582,27 +3437,27 @@
       <c r="E82" s="5"/>
       <c r="F82" s="6"/>
     </row>
-    <row r="83" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
       <c r="F83" s="6"/>
     </row>
-    <row r="84" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="84" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <conditionalFormatting sqref="C2:C9">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10:D1048576 C1">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>